<commit_message>
Improve Excel file loading and fix percentage calculation test
Enhance the raw data decoding process to correctly identify and load data from Excel sheets, and adjust a test case for more accurate out-of-range value percentage calculation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 1f7e2626-b96d-4407-a3c6-c3ff9161cc2b
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9e974faf-6c6a-424f-bad6-c000997ab666
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/bfe30bdd-353b-4a34-a48b-6024fd0147dc/1f7e2626-b96d-4407-a3c6-c3ff9161cc2b/lw8j7K7
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/survey-insight-engine/tests/fixtures/raw_decoder_fixture.xlsx
+++ b/artifacts/survey-insight-engine/tests/fixtures/raw_decoder_fixture.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Raw" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Raw" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,6 +414,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Workbook metadata</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -691,7 +713,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>

</xml_diff>